<commit_message>
Add Nifty 100 corporate tear sheets and script updates
</commit_message>
<xml_diff>
--- a/output/valuation_summary.xlsx
+++ b/output/valuation_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,47 +417,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>free_cash_flow_cr</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>earnings_per_share</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>book_value_per_share</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>FCF Yield Score</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>PE Flag</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Valuation</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>composite_score</t>
         </is>
@@ -618,7 +606,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>73.39865162986888</v>
+        <v>73.39865162986887</v>
       </c>
     </row>
     <row r="6">
@@ -727,7 +715,7 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>72.22100379305637</v>
+        <v>72.22100379305638</v>
       </c>
     </row>
     <row r="9">
@@ -1083,7 +1071,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>58.41584158415842</v>
+        <v>58.41584158415841</v>
       </c>
     </row>
     <row r="19">
@@ -1330,7 +1318,7 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>50.43077753153465</v>
+        <v>50.43077753153466</v>
       </c>
     </row>
     <row r="26">
@@ -1365,7 +1353,7 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>50.33176763054457</v>
+        <v>50.33176763054456</v>
       </c>
     </row>
     <row r="27">
@@ -1610,7 +1598,7 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>49.53968842262378</v>
+        <v>49.53968842262377</v>
       </c>
     </row>
     <row r="34">
@@ -1855,7 +1843,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>48.64859931371289</v>
+        <v>48.64859931371288</v>
       </c>
     </row>
     <row r="41">
@@ -2240,7 +2228,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>47.46048050183168</v>
+        <v>47.46048050183169</v>
       </c>
     </row>
     <row r="52">
@@ -2391,7 +2379,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Asian Paints
+          <t>Asian Paints
 Indian Multi-National Paint and Coating Manufacturing Company</t>
         </is>
       </c>
@@ -2486,7 +2474,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>46.86642109589111</v>
+        <v>46.8664210958911</v>
       </c>
     </row>
     <row r="59">
@@ -2624,7 +2612,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>46.37137159094061</v>
+        <v>46.3713715909406</v>
       </c>
     </row>
     <row r="63">
@@ -2694,7 +2682,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>46.27236168995051</v>
+        <v>46.2723616899505</v>
       </c>
     </row>
     <row r="65">
@@ -2834,7 +2822,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>45.6783022840099</v>
+        <v>45.67830228400991</v>
       </c>
     </row>
     <row r="69">
@@ -3079,7 +3067,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>45.08424287806932</v>
+        <v>45.08424287806931</v>
       </c>
     </row>
     <row r="76">
@@ -3114,7 +3102,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>44.98523297707922</v>
+        <v>44.98523297707921</v>
       </c>
     </row>
     <row r="77">
@@ -3300,7 +3288,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Apollo Hospitals
+          <t>Apollo Hospitals
 Chain of Indian private hospitals</t>
         </is>
       </c>
@@ -3500,7 +3488,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>43.89612406618814</v>
+        <v>43.89612406618813</v>
       </c>
     </row>
     <row r="88">
@@ -3708,7 +3696,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>43.30206466024754</v>
+        <v>43.30206466024753</v>
       </c>
     </row>
     <row r="94">
@@ -3813,7 +3801,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>42.70800525430693</v>
+        <v>42.70800525430694</v>
       </c>
     </row>
     <row r="97">

</xml_diff>

<commit_message>
update all the modified files
</commit_message>
<xml_diff>
--- a/output/valuation_summary.xlsx
+++ b/output/valuation_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,47 +429,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>free_cash_flow_cr</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>earnings_per_share</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>book_value_per_share</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>FCF Yield Score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>PE Flag</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valuation</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>composite_score</t>
         </is>
@@ -606,7 +618,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>73.39865162986887</v>
+        <v>73.39865162986888</v>
       </c>
     </row>
     <row r="6">
@@ -715,7 +727,7 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>72.22100379305638</v>
+        <v>72.22100379305637</v>
       </c>
     </row>
     <row r="9">
@@ -1071,7 +1083,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>58.41584158415841</v>
+        <v>58.41584158415842</v>
       </c>
     </row>
     <row r="19">
@@ -1318,7 +1330,7 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>50.43077753153466</v>
+        <v>50.43077753153465</v>
       </c>
     </row>
     <row r="26">
@@ -1353,7 +1365,7 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>50.33176763054456</v>
+        <v>50.33176763054457</v>
       </c>
     </row>
     <row r="27">
@@ -1598,7 +1610,7 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>49.53968842262377</v>
+        <v>49.53968842262378</v>
       </c>
     </row>
     <row r="34">
@@ -1843,7 +1855,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>48.64859931371288</v>
+        <v>48.64859931371289</v>
       </c>
     </row>
     <row r="41">
@@ -2228,7 +2240,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>47.46048050183169</v>
+        <v>47.46048050183168</v>
       </c>
     </row>
     <row r="52">
@@ -2379,7 +2391,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Asian Paints
+          <t>Asian Paints
 Indian Multi-National Paint and Coating Manufacturing Company</t>
         </is>
       </c>
@@ -2474,7 +2486,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>46.8664210958911</v>
+        <v>46.86642109589111</v>
       </c>
     </row>
     <row r="59">
@@ -2612,7 +2624,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>46.3713715909406</v>
+        <v>46.37137159094061</v>
       </c>
     </row>
     <row r="63">
@@ -2682,7 +2694,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>46.2723616899505</v>
+        <v>46.27236168995051</v>
       </c>
     </row>
     <row r="65">
@@ -2822,7 +2834,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>45.67830228400991</v>
+        <v>45.6783022840099</v>
       </c>
     </row>
     <row r="69">
@@ -3067,7 +3079,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>45.08424287806931</v>
+        <v>45.08424287806932</v>
       </c>
     </row>
     <row r="76">
@@ -3102,7 +3114,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>44.98523297707921</v>
+        <v>44.98523297707922</v>
       </c>
     </row>
     <row r="77">
@@ -3288,7 +3300,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Apollo Hospitals
+          <t>Apollo Hospitals
 Chain of Indian private hospitals</t>
         </is>
       </c>
@@ -3488,7 +3500,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>43.89612406618813</v>
+        <v>43.89612406618814</v>
       </c>
     </row>
     <row r="88">
@@ -3696,7 +3708,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>43.30206466024753</v>
+        <v>43.30206466024754</v>
       </c>
     </row>
     <row r="94">
@@ -3801,7 +3813,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>42.70800525430694</v>
+        <v>42.70800525430693</v>
       </c>
     </row>
     <row r="97">

</xml_diff>